<commit_message>
updated the data dictionary part1
</commit_message>
<xml_diff>
--- a/docs/Data_Dictionary.xlsx
+++ b/docs/Data_Dictionary.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HomePC\Desktop\classification_project\docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35FEDFA3-164A-4A0E-BB52-34D5CF885B18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,271 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="86">
+  <si>
+    <t>Column Name</t>
+  </si>
+  <si>
+    <t>Data Type</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Business Meaning</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>SK_ID_CURR</t>
+  </si>
+  <si>
+    <t>int64</t>
+  </si>
+  <si>
+    <t>Identifier</t>
+  </si>
+  <si>
+    <t>Unique identifier assigned to each customer/application record</t>
+  </si>
+  <si>
+    <t>Not a predictive feature</t>
+  </si>
+  <si>
+    <t>TARGET</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>Indicates whether the applicant experienced payment difficulties/default</t>
+  </si>
+  <si>
+    <t>0 = no payment difficulties, 1 = payment difficulties</t>
+  </si>
+  <si>
+    <t>NAME_CONTRACT_TYPE</t>
+  </si>
+  <si>
+    <t>object</t>
+  </si>
+  <si>
+    <t>Feature</t>
+  </si>
+  <si>
+    <t>Type of loan contract associated with the application</t>
+  </si>
+  <si>
+    <t>Categorical feature</t>
+  </si>
+  <si>
+    <t>CODE_GENDER</t>
+  </si>
+  <si>
+    <t>Gender of the applicant</t>
+  </si>
+  <si>
+    <t>FLAG_OWN_CAR</t>
+  </si>
+  <si>
+    <t>Indicates whether the applicant owns a car</t>
+  </si>
+  <si>
+    <t>Binary categorical feature</t>
+  </si>
+  <si>
+    <t>FLAG_OWN_REALTY</t>
+  </si>
+  <si>
+    <t>Indicates whether the applicant owns real estate/property</t>
+  </si>
+  <si>
+    <t>CNT_CHILDREN</t>
+  </si>
+  <si>
+    <t>Number of children of the applicant</t>
+  </si>
+  <si>
+    <t>Count variable</t>
+  </si>
+  <si>
+    <t>AMT_INCOME_TOTAL</t>
+  </si>
+  <si>
+    <t>float64</t>
+  </si>
+  <si>
+    <t>Total income of the applicant</t>
+  </si>
+  <si>
+    <t>Monetary value</t>
+  </si>
+  <si>
+    <t>AMT_CREDIT</t>
+  </si>
+  <si>
+    <t>Amount of credit/loan granted to the applicant</t>
+  </si>
+  <si>
+    <t>AMT_ANNUITY</t>
+  </si>
+  <si>
+    <t>Periodic loan repayment amount associated with the application</t>
+  </si>
+  <si>
+    <t>AMT_GOODS_PRICE</t>
+  </si>
+  <si>
+    <t>Price of the goods or item being financed</t>
+  </si>
+  <si>
+    <t>NAME_TYPE_SUITE</t>
+  </si>
+  <si>
+    <t>Type of person who accompanied the applicant when applying for the loan</t>
+  </si>
+  <si>
+    <t>NAME_INCOME_TYPE</t>
+  </si>
+  <si>
+    <t>Type/source of income or employment status of the applicant</t>
+  </si>
+  <si>
+    <t>NAME_EDUCATION_TYPE</t>
+  </si>
+  <si>
+    <t>Education or qualification level of the applicant</t>
+  </si>
+  <si>
+    <t>NAME_FAMILY_STATUS</t>
+  </si>
+  <si>
+    <t>Marital/family status of the applicant</t>
+  </si>
+  <si>
+    <t>NAME_HOUSING_TYPE</t>
+  </si>
+  <si>
+    <t>Type of housing/accommodation in which the applicant lives</t>
+  </si>
+  <si>
+    <t>REGION_POPULATION_RELATIVE</t>
+  </si>
+  <si>
+    <t>Normalized measure of the population density of the applicant's region</t>
+  </si>
+  <si>
+    <t>Relative regional population measure</t>
+  </si>
+  <si>
+    <t>DAYS_BIRTH</t>
+  </si>
+  <si>
+    <t>Number of days between the applicant's birth date and the loan application date</t>
+  </si>
+  <si>
+    <t>Negative values are expected; can be transformed into age</t>
+  </si>
+  <si>
+    <t>DAYS_EMPLOYED</t>
+  </si>
+  <si>
+    <t>Duration of the applicant's employment before the loan application, measured in days</t>
+  </si>
+  <si>
+    <t>Negative values are expected; 365243 is a special/unknown value</t>
+  </si>
+  <si>
+    <t>DAYS_REGISTRATION</t>
+  </si>
+  <si>
+    <t>Number of days between the applicant's registration date and the loan application date</t>
+  </si>
+  <si>
+    <t>Negative values indicate registration occurred before the application</t>
+  </si>
+  <si>
+    <t>DAYS_ID_PUBLISH</t>
+  </si>
+  <si>
+    <t>Number of days between the applicant's ID document publication/issuance date and the loan application date</t>
+  </si>
+  <si>
+    <t>Negative values indicate the ID was published before the application</t>
+  </si>
+  <si>
+    <t>OWN_CAR_AGE</t>
+  </si>
+  <si>
+    <t>Age of the car owned by the applicant, measured in years</t>
+  </si>
+  <si>
+    <t>Represents vehicle age, not duration of ownership</t>
+  </si>
+  <si>
+    <t>FLAG_MOBIL</t>
+  </si>
+  <si>
+    <t>Indicates whether the applicant has/provides a mobile phone number</t>
+  </si>
+  <si>
+    <t>Binary indicator</t>
+  </si>
+  <si>
+    <t>FLAG_EMP_PHONE</t>
+  </si>
+  <si>
+    <t>Indicates whether the applicant has/provides a work/employment phone number</t>
+  </si>
+  <si>
+    <t>FLAG_WORK_PHONE</t>
+  </si>
+  <si>
+    <t>Indicates whether a work phone number is available/provided</t>
+  </si>
+  <si>
+    <t>FLAG_CONT_MOBILE</t>
+  </si>
+  <si>
+    <t>Indicates whether the applicant is reachable through their mobile phone</t>
+  </si>
+  <si>
+    <t>OCCUPATION_TYPE</t>
+  </si>
+  <si>
+    <t>Occupation type of the applicant</t>
+  </si>
+  <si>
+    <t>Categorical feature; contains missing values</t>
+  </si>
+  <si>
+    <t>CNT_FAM_MEMBERS</t>
+  </si>
+  <si>
+    <t>Number of family members associated with the applicant</t>
+  </si>
+  <si>
+    <t>FLAG_PHONE</t>
+  </si>
+  <si>
+    <t>Indicates whether the applicant has provided a phone number</t>
+  </si>
+  <si>
+    <t>Binary indicator; 1 = yes, 0 = no</t>
+  </si>
+  <si>
+    <t>FLAG_EMAIL</t>
+  </si>
+  <si>
+    <t>Indicates whether the applicant has provided an email address</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -330,10 +599,543 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="27.90625" customWidth="1"/>
+    <col min="4" max="4" width="74.6328125" customWidth="1"/>
+    <col min="5" max="5" width="43.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" t="s">
+        <v>48</v>
+      </c>
+      <c r="E17" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" t="s">
+        <v>50</v>
+      </c>
+      <c r="E18" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" t="s">
+        <v>53</v>
+      </c>
+      <c r="E19" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" t="s">
+        <v>56</v>
+      </c>
+      <c r="E20" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" t="s">
+        <v>59</v>
+      </c>
+      <c r="E21" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>64</v>
+      </c>
+      <c r="B23" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" t="s">
+        <v>65</v>
+      </c>
+      <c r="E23" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>67</v>
+      </c>
+      <c r="B24" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" t="s">
+        <v>68</v>
+      </c>
+      <c r="E24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>70</v>
+      </c>
+      <c r="B25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" t="s">
+        <v>71</v>
+      </c>
+      <c r="E25" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>72</v>
+      </c>
+      <c r="B26" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" t="s">
+        <v>73</v>
+      </c>
+      <c r="E26" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>74</v>
+      </c>
+      <c r="B27" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" t="s">
+        <v>75</v>
+      </c>
+      <c r="E27" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>81</v>
+      </c>
+      <c r="B28" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" t="s">
+        <v>82</v>
+      </c>
+      <c r="E28" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>84</v>
+      </c>
+      <c r="B29" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" t="s">
+        <v>85</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>76</v>
+      </c>
+      <c r="B30" t="s">
+        <v>15</v>
+      </c>
+      <c r="C30" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30" t="s">
+        <v>77</v>
+      </c>
+      <c r="E30" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>79</v>
+      </c>
+      <c r="B31" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" t="s">
+        <v>80</v>
+      </c>
+      <c r="E31" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>